<commit_message>
Update Pertanggal 16 April 2026 18:19 WIB
</commit_message>
<xml_diff>
--- a/Documentation/Documents/SQL Function Test/SchData-OLTP-Master.Func_General_GetBusinessDocumentTypeIDByName.xlsx
+++ b/Documentation/Documents/SQL Function Test/SchData-OLTP-Master.Func_General_GetBusinessDocumentTypeIDByName.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="Result" sheetId="1" r:id="rId1"/>
@@ -457,48 +457,18 @@
   <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyFill="1" applyBorder="1"/>
@@ -524,6 +494,36 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma [0]" xfId="1" builtinId="6"/>
@@ -845,805 +845,836 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:11" s="31" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="14" t="s">
+    <row r="2" spans="2:11" s="21" customFormat="1" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="D2" s="14" t="s">
+      <c r="C2" s="40"/>
+      <c r="D2" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="E2" s="15"/>
-      <c r="F2" s="14" t="s">
+      <c r="E2" s="40"/>
+      <c r="F2" s="39" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="15"/>
-      <c r="I2" s="32" t="s">
+      <c r="G2" s="40"/>
+      <c r="I2" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="J2" s="33" t="s">
+      <c r="J2" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="K2" s="34" t="s">
+      <c r="K2" s="24" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B3" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="23">
+      <c r="B3" s="35" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="36">
         <v>4000000000359</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="23">
+      <c r="E3" s="36">
         <v>46000000000009</v>
       </c>
-      <c r="F3" s="24" t="s">
+      <c r="F3" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="25">
+      <c r="G3" s="15">
         <v>77000000000057</v>
       </c>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B4" s="2"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="6" t="s">
+      <c r="B4" s="31"/>
+      <c r="C4" s="33"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="33"/>
+      <c r="F4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="7">
+      <c r="G4" s="3">
         <v>77000000000041</v>
       </c>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B5" s="2"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="6" t="s">
+      <c r="B5" s="31"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="31"/>
+      <c r="E5" s="33"/>
+      <c r="F5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="7">
+      <c r="G5" s="3">
         <v>77000000000045</v>
       </c>
     </row>
     <row r="6" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B6" s="2"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="2" t="s">
+      <c r="B6" s="31"/>
+      <c r="C6" s="33"/>
+      <c r="D6" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="3">
+      <c r="E6" s="33">
         <v>46000000000033</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="7">
+      <c r="G6" s="3">
         <v>77000000000057</v>
       </c>
     </row>
     <row r="7" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B7" s="2"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="6" t="s">
+      <c r="B7" s="31"/>
+      <c r="C7" s="33"/>
+      <c r="D7" s="31"/>
+      <c r="E7" s="33"/>
+      <c r="F7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G7" s="7">
+      <c r="G7" s="3">
         <v>77000000000041</v>
       </c>
     </row>
     <row r="8" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="4"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="8" t="s">
+      <c r="B8" s="32"/>
+      <c r="C8" s="34"/>
+      <c r="D8" s="32"/>
+      <c r="E8" s="34"/>
+      <c r="F8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G8" s="9">
+      <c r="G8" s="5">
         <v>77000000000045</v>
       </c>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="36">
         <v>4000000000029</v>
       </c>
-      <c r="D9" s="22" t="s">
+      <c r="D9" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="E9" s="23">
+      <c r="E9" s="36">
         <v>46000000000009</v>
       </c>
-      <c r="F9" s="24" t="s">
+      <c r="F9" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="25">
+      <c r="G9" s="15">
         <v>77000000000057</v>
       </c>
-      <c r="I9" s="16" t="b">
+      <c r="I9" s="8" t="b">
         <v>1</v>
       </c>
-      <c r="J9" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="K9" s="17" t="b">
+      <c r="J9" s="25" t="b">
+        <v>0</v>
+      </c>
+      <c r="K9" s="9" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="10" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B10" s="2"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="6" t="s">
+      <c r="B10" s="31"/>
+      <c r="C10" s="33"/>
+      <c r="D10" s="31"/>
+      <c r="E10" s="33"/>
+      <c r="F10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="7">
+      <c r="G10" s="3">
         <v>77000000000041</v>
       </c>
-      <c r="I10" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J10" s="36" t="b">
-        <v>0</v>
-      </c>
-      <c r="K10" s="19" t="b">
+      <c r="I10" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J10" s="26" t="b">
+        <v>0</v>
+      </c>
+      <c r="K10" s="11" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B11" s="2"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="6" t="s">
+      <c r="B11" s="31"/>
+      <c r="C11" s="33"/>
+      <c r="D11" s="31"/>
+      <c r="E11" s="33"/>
+      <c r="F11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G11" s="7">
+      <c r="G11" s="3">
         <v>77000000000045</v>
       </c>
-      <c r="I11" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J11" s="36" t="b">
-        <v>0</v>
-      </c>
-      <c r="K11" s="19" t="b">
+      <c r="I11" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J11" s="26" t="b">
+        <v>0</v>
+      </c>
+      <c r="K11" s="11" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B12" s="2"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="2" t="s">
+      <c r="B12" s="31"/>
+      <c r="C12" s="33"/>
+      <c r="D12" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="E12" s="3">
+      <c r="E12" s="33">
         <v>46000000000033</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G12" s="7">
+      <c r="G12" s="3">
         <v>77000000000057</v>
       </c>
-      <c r="I12" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J12" s="36" t="b">
+      <c r="I12" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J12" s="26" t="b">
         <v>1</v>
       </c>
-      <c r="K12" s="19" t="b">
+      <c r="K12" s="11" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="13" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B13" s="2"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="6" t="s">
+      <c r="B13" s="31"/>
+      <c r="C13" s="33"/>
+      <c r="D13" s="31"/>
+      <c r="E13" s="33"/>
+      <c r="F13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G13" s="7">
+      <c r="G13" s="3">
         <v>77000000000041</v>
       </c>
-      <c r="I13" s="18" t="b">
+      <c r="I13" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J13" s="36" t="b">
-        <v>0</v>
-      </c>
-      <c r="K13" s="19" t="b">
+      <c r="J13" s="26" t="b">
+        <v>0</v>
+      </c>
+      <c r="K13" s="11" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="4"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="8" t="s">
+      <c r="B14" s="32"/>
+      <c r="C14" s="34"/>
+      <c r="D14" s="32"/>
+      <c r="E14" s="34"/>
+      <c r="F14" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G14" s="9">
+      <c r="G14" s="5">
         <v>77000000000045</v>
       </c>
-      <c r="I14" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="J14" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="K14" s="21" t="b">
+      <c r="I14" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J14" s="27" t="b">
+        <v>0</v>
+      </c>
+      <c r="K14" s="13" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="35" t="s">
         <v>2</v>
       </c>
-      <c r="C15" s="23">
+      <c r="C15" s="36">
         <v>4000000000534</v>
       </c>
-      <c r="D15" s="22" t="s">
+      <c r="D15" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="E15" s="23">
+      <c r="E15" s="36">
         <v>46000000000009</v>
       </c>
-      <c r="F15" s="24" t="s">
+      <c r="F15" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="G15" s="25">
+      <c r="G15" s="15">
         <v>77000000000057</v>
       </c>
-      <c r="I15" s="16" t="b">
-        <v>0</v>
-      </c>
-      <c r="J15" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="K15" s="17" t="b">
+      <c r="I15" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J15" s="25" t="b">
+        <v>0</v>
+      </c>
+      <c r="K15" s="9" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B16" s="2"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="6" t="s">
+      <c r="B16" s="31"/>
+      <c r="C16" s="33"/>
+      <c r="D16" s="31"/>
+      <c r="E16" s="33"/>
+      <c r="F16" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G16" s="7">
+      <c r="G16" s="3">
         <v>77000000000041</v>
       </c>
-      <c r="I16" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J16" s="36" t="b">
-        <v>0</v>
-      </c>
-      <c r="K16" s="19" t="b">
+      <c r="I16" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J16" s="26" t="b">
+        <v>0</v>
+      </c>
+      <c r="K16" s="11" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B17" s="2"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="6" t="s">
+      <c r="B17" s="31"/>
+      <c r="C17" s="33"/>
+      <c r="D17" s="31"/>
+      <c r="E17" s="33"/>
+      <c r="F17" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="7">
+      <c r="G17" s="3">
         <v>77000000000045</v>
       </c>
-      <c r="I17" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J17" s="36" t="b">
-        <v>0</v>
-      </c>
-      <c r="K17" s="19" t="b">
+      <c r="I17" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J17" s="26" t="b">
+        <v>0</v>
+      </c>
+      <c r="K17" s="11" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B18" s="2"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="2" t="s">
+      <c r="B18" s="31"/>
+      <c r="C18" s="33"/>
+      <c r="D18" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="E18" s="3">
+      <c r="E18" s="33">
         <v>46000000000033</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="F18" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G18" s="7">
+      <c r="G18" s="3">
         <v>77000000000057</v>
       </c>
-      <c r="I18" s="18" t="b">
+      <c r="I18" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J18" s="36" t="b">
-        <v>0</v>
-      </c>
-      <c r="K18" s="19" t="b">
+      <c r="J18" s="26" t="b">
+        <v>0</v>
+      </c>
+      <c r="K18" s="11" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="19" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B19" s="2"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="6" t="s">
+      <c r="B19" s="31"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="31"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G19" s="7">
+      <c r="G19" s="3">
         <v>77000000000041</v>
       </c>
-      <c r="I19" s="18" t="b">
+      <c r="I19" s="10" t="b">
         <v>1</v>
       </c>
-      <c r="J19" s="36" t="b">
-        <v>0</v>
-      </c>
-      <c r="K19" s="19" t="b">
+      <c r="J19" s="26" t="b">
+        <v>0</v>
+      </c>
+      <c r="K19" s="11" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="20" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="4"/>
-      <c r="C20" s="5"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="5"/>
-      <c r="F20" s="8" t="s">
+      <c r="B20" s="32"/>
+      <c r="C20" s="34"/>
+      <c r="D20" s="32"/>
+      <c r="E20" s="34"/>
+      <c r="F20" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G20" s="9">
+      <c r="G20" s="5">
         <v>77000000000045</v>
       </c>
-      <c r="I20" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="J20" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="K20" s="21" t="b">
+      <c r="I20" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J20" s="27" t="b">
+        <v>0</v>
+      </c>
+      <c r="K20" s="13" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="C21" s="23">
+      <c r="C21" s="36">
         <v>4000000000577</v>
       </c>
-      <c r="D21" s="22" t="s">
+      <c r="D21" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="E21" s="23">
+      <c r="E21" s="36">
         <v>46000000000009</v>
       </c>
-      <c r="F21" s="24" t="s">
+      <c r="F21" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="G21" s="25">
+      <c r="G21" s="15">
         <v>77000000000057</v>
       </c>
-      <c r="I21" s="16" t="b">
-        <v>0</v>
-      </c>
-      <c r="J21" s="35" t="b">
-        <v>0</v>
-      </c>
-      <c r="K21" s="27" t="b">
+      <c r="I21" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J21" s="25" t="b">
+        <v>0</v>
+      </c>
+      <c r="K21" s="17" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B22" s="2"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="6" t="s">
+      <c r="B22" s="31"/>
+      <c r="C22" s="33"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="33"/>
+      <c r="F22" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G22" s="7">
+      <c r="G22" s="3">
         <v>77000000000041</v>
       </c>
-      <c r="I22" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J22" s="36" t="b">
+      <c r="I22" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J22" s="26" t="b">
         <v>1</v>
       </c>
-      <c r="K22" s="26" t="b">
+      <c r="K22" s="16" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="23" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B23" s="2"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="6" t="s">
+      <c r="B23" s="31"/>
+      <c r="C23" s="33"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="33"/>
+      <c r="F23" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G23" s="7">
+      <c r="G23" s="3">
         <v>77000000000045</v>
       </c>
-      <c r="I23" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J23" s="36" t="b">
-        <v>0</v>
-      </c>
-      <c r="K23" s="26" t="b">
+      <c r="I23" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J23" s="26" t="b">
+        <v>0</v>
+      </c>
+      <c r="K23" s="16" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B24" s="2"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="2" t="s">
+      <c r="B24" s="31"/>
+      <c r="C24" s="33"/>
+      <c r="D24" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="E24" s="3">
+      <c r="E24" s="33">
         <v>46000000000033</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="F24" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G24" s="7">
+      <c r="G24" s="3">
         <v>77000000000057</v>
       </c>
-      <c r="I24" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J24" s="36" t="b">
-        <v>0</v>
-      </c>
-      <c r="K24" s="19" t="b">
+      <c r="I24" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J24" s="26" t="b">
+        <v>0</v>
+      </c>
+      <c r="K24" s="11" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B25" s="2"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="6" t="s">
+      <c r="B25" s="31"/>
+      <c r="C25" s="33"/>
+      <c r="D25" s="31"/>
+      <c r="E25" s="33"/>
+      <c r="F25" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G25" s="7">
+      <c r="G25" s="3">
         <v>77000000000041</v>
       </c>
-      <c r="I25" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J25" s="36" t="b">
+      <c r="I25" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J25" s="26" t="b">
         <v>1</v>
       </c>
-      <c r="K25" s="19" t="b">
+      <c r="K25" s="11" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="26" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="4"/>
-      <c r="C26" s="5"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="5"/>
-      <c r="F26" s="8" t="s">
+      <c r="B26" s="32"/>
+      <c r="C26" s="34"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="34"/>
+      <c r="F26" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G26" s="9">
+      <c r="G26" s="5">
         <v>77000000000045</v>
       </c>
-      <c r="I26" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="J26" s="37" t="b">
-        <v>0</v>
-      </c>
-      <c r="K26" s="21" t="b">
+      <c r="I26" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J26" s="27" t="b">
+        <v>0</v>
+      </c>
+      <c r="K26" s="13" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B27" s="22" t="s">
+      <c r="B27" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="C27" s="23">
+      <c r="C27" s="36">
         <v>4000000000495</v>
       </c>
-      <c r="D27" s="22" t="s">
+      <c r="D27" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="E27" s="23">
+      <c r="E27" s="36">
         <v>46000000000009</v>
       </c>
-      <c r="F27" s="24" t="s">
+      <c r="F27" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="G27" s="25">
+      <c r="G27" s="15">
         <v>77000000000057</v>
       </c>
-      <c r="I27" s="29" t="b">
-        <v>0</v>
-      </c>
-      <c r="J27" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="K27" s="27" t="b">
+      <c r="I27" s="19" t="b">
+        <v>0</v>
+      </c>
+      <c r="J27" s="28" t="b">
+        <v>0</v>
+      </c>
+      <c r="K27" s="17" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B28" s="2"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="6" t="s">
+      <c r="B28" s="31"/>
+      <c r="C28" s="33"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="33"/>
+      <c r="F28" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G28" s="7">
+      <c r="G28" s="3">
         <v>77000000000041</v>
       </c>
-      <c r="I28" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J28" s="39" t="b">
-        <v>0</v>
-      </c>
-      <c r="K28" s="26" t="b">
+      <c r="I28" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J28" s="29" t="b">
+        <v>0</v>
+      </c>
+      <c r="K28" s="16" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B29" s="2"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="6" t="s">
+      <c r="B29" s="31"/>
+      <c r="C29" s="33"/>
+      <c r="D29" s="31"/>
+      <c r="E29" s="33"/>
+      <c r="F29" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G29" s="7">
+      <c r="G29" s="3">
         <v>77000000000045</v>
       </c>
-      <c r="I29" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J29" s="39" t="b">
-        <v>0</v>
-      </c>
-      <c r="K29" s="26" t="b">
+      <c r="I29" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J29" s="29" t="b">
+        <v>0</v>
+      </c>
+      <c r="K29" s="16" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B30" s="2"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="2" t="s">
+      <c r="B30" s="31"/>
+      <c r="C30" s="33"/>
+      <c r="D30" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="E30" s="3">
+      <c r="E30" s="33">
         <v>46000000000033</v>
       </c>
-      <c r="F30" s="6" t="s">
+      <c r="F30" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G30" s="7">
+      <c r="G30" s="3">
         <v>77000000000057</v>
       </c>
-      <c r="I30" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J30" s="39" t="b">
-        <v>0</v>
-      </c>
-      <c r="K30" s="26" t="b">
+      <c r="I30" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J30" s="29" t="b">
+        <v>0</v>
+      </c>
+      <c r="K30" s="16" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B31" s="2"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="2"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="6" t="s">
+      <c r="B31" s="31"/>
+      <c r="C31" s="33"/>
+      <c r="D31" s="31"/>
+      <c r="E31" s="33"/>
+      <c r="F31" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G31" s="7">
+      <c r="G31" s="3">
         <v>77000000000041</v>
       </c>
-      <c r="I31" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J31" s="39" t="b">
-        <v>0</v>
-      </c>
-      <c r="K31" s="26" t="b">
+      <c r="I31" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J31" s="29" t="b">
+        <v>0</v>
+      </c>
+      <c r="K31" s="16" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="32" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="4"/>
-      <c r="C32" s="5"/>
-      <c r="D32" s="4"/>
-      <c r="E32" s="5"/>
-      <c r="F32" s="8" t="s">
+      <c r="B32" s="32"/>
+      <c r="C32" s="34"/>
+      <c r="D32" s="32"/>
+      <c r="E32" s="34"/>
+      <c r="F32" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G32" s="9">
+      <c r="G32" s="5">
         <v>77000000000045</v>
       </c>
-      <c r="I32" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="J32" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="K32" s="30" t="b">
+      <c r="I32" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J32" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="K32" s="20" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="33" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B33" s="10" t="s">
+      <c r="B33" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="C33" s="11">
+      <c r="C33" s="38">
         <v>4000000000486</v>
       </c>
-      <c r="D33" s="10" t="s">
+      <c r="D33" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="E33" s="11">
+      <c r="E33" s="38">
         <v>46000000000009</v>
       </c>
-      <c r="F33" s="12" t="s">
+      <c r="F33" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G33" s="13">
+      <c r="G33" s="7">
         <v>77000000000057</v>
       </c>
-      <c r="I33" s="28" t="b">
-        <v>0</v>
-      </c>
-      <c r="J33" s="38" t="b">
-        <v>0</v>
-      </c>
-      <c r="K33" s="26" t="b">
+      <c r="I33" s="18" t="b">
+        <v>0</v>
+      </c>
+      <c r="J33" s="28" t="b">
+        <v>0</v>
+      </c>
+      <c r="K33" s="16" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="34" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B34" s="2"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="3"/>
-      <c r="F34" s="6" t="s">
+      <c r="B34" s="31"/>
+      <c r="C34" s="33"/>
+      <c r="D34" s="31"/>
+      <c r="E34" s="33"/>
+      <c r="F34" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G34" s="7">
+      <c r="G34" s="3">
         <v>77000000000041</v>
       </c>
-      <c r="I34" s="28" t="b">
+      <c r="I34" s="18" t="b">
         <v>1</v>
       </c>
-      <c r="J34" s="39" t="b">
-        <v>0</v>
-      </c>
-      <c r="K34" s="26" t="b">
+      <c r="J34" s="29" t="b">
+        <v>0</v>
+      </c>
+      <c r="K34" s="16" t="b">
         <v>1</v>
       </c>
     </row>
     <row r="35" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B35" s="2"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="6" t="s">
+      <c r="B35" s="31"/>
+      <c r="C35" s="33"/>
+      <c r="D35" s="31"/>
+      <c r="E35" s="33"/>
+      <c r="F35" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G35" s="7">
+      <c r="G35" s="3">
         <v>77000000000045</v>
       </c>
-      <c r="I35" s="28" t="b">
-        <v>0</v>
-      </c>
-      <c r="J35" s="39" t="b">
-        <v>0</v>
-      </c>
-      <c r="K35" s="26" t="b">
+      <c r="I35" s="18" t="b">
+        <v>0</v>
+      </c>
+      <c r="J35" s="29" t="b">
+        <v>0</v>
+      </c>
+      <c r="K35" s="16" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="36" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B36" s="2"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="2" t="s">
+      <c r="B36" s="31"/>
+      <c r="C36" s="33"/>
+      <c r="D36" s="31" t="s">
         <v>8</v>
       </c>
-      <c r="E36" s="3">
+      <c r="E36" s="33">
         <v>46000000000033</v>
       </c>
-      <c r="F36" s="6" t="s">
+      <c r="F36" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="G36" s="7">
+      <c r="G36" s="3">
         <v>77000000000057</v>
       </c>
-      <c r="I36" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J36" s="39" t="b">
-        <v>0</v>
-      </c>
-      <c r="K36" s="26" t="b">
+      <c r="I36" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J36" s="29" t="b">
+        <v>0</v>
+      </c>
+      <c r="K36" s="16" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="37" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B37" s="2"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="6" t="s">
+      <c r="B37" s="31"/>
+      <c r="C37" s="33"/>
+      <c r="D37" s="31"/>
+      <c r="E37" s="33"/>
+      <c r="F37" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="G37" s="7">
+      <c r="G37" s="3">
         <v>77000000000041</v>
       </c>
-      <c r="I37" s="18" t="b">
-        <v>0</v>
-      </c>
-      <c r="J37" s="39" t="b">
-        <v>0</v>
-      </c>
-      <c r="K37" s="26" t="b">
+      <c r="I37" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="J37" s="29" t="b">
+        <v>0</v>
+      </c>
+      <c r="K37" s="16" t="b">
         <v>0</v>
       </c>
     </row>
     <row r="38" spans="2:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="4"/>
-      <c r="C38" s="5"/>
-      <c r="D38" s="4"/>
-      <c r="E38" s="5"/>
-      <c r="F38" s="8" t="s">
+      <c r="B38" s="32"/>
+      <c r="C38" s="34"/>
+      <c r="D38" s="32"/>
+      <c r="E38" s="34"/>
+      <c r="F38" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G38" s="9">
+      <c r="G38" s="5">
         <v>77000000000045</v>
       </c>
-      <c r="I38" s="20" t="b">
-        <v>0</v>
-      </c>
-      <c r="J38" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="K38" s="30" t="b">
+      <c r="I38" s="12" t="b">
+        <v>0</v>
+      </c>
+      <c r="J38" s="30" t="b">
+        <v>0</v>
+      </c>
+      <c r="K38" s="20" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="39">
+    <mergeCell ref="D6:D8"/>
+    <mergeCell ref="E6:E8"/>
+    <mergeCell ref="B3:B8"/>
+    <mergeCell ref="C3:C8"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="E3:E5"/>
+    <mergeCell ref="E9:E11"/>
+    <mergeCell ref="D12:D14"/>
+    <mergeCell ref="E12:E14"/>
+    <mergeCell ref="D15:D17"/>
+    <mergeCell ref="E15:E17"/>
+    <mergeCell ref="B27:B32"/>
+    <mergeCell ref="C27:C32"/>
+    <mergeCell ref="B33:B38"/>
+    <mergeCell ref="C33:C38"/>
+    <mergeCell ref="D9:D11"/>
+    <mergeCell ref="B9:B14"/>
+    <mergeCell ref="C9:C14"/>
+    <mergeCell ref="B15:B20"/>
+    <mergeCell ref="C15:C20"/>
+    <mergeCell ref="B21:B26"/>
+    <mergeCell ref="C21:C26"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:E20"/>
+    <mergeCell ref="D21:D23"/>
+    <mergeCell ref="E21:E23"/>
+    <mergeCell ref="D24:D26"/>
+    <mergeCell ref="E24:E26"/>
     <mergeCell ref="D36:D38"/>
     <mergeCell ref="E36:E38"/>
     <mergeCell ref="D27:D29"/>
@@ -1652,37 +1683,6 @@
     <mergeCell ref="E30:E32"/>
     <mergeCell ref="D33:D35"/>
     <mergeCell ref="E33:E35"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:E20"/>
-    <mergeCell ref="D21:D23"/>
-    <mergeCell ref="E21:E23"/>
-    <mergeCell ref="D24:D26"/>
-    <mergeCell ref="E24:E26"/>
-    <mergeCell ref="B27:B32"/>
-    <mergeCell ref="C27:C32"/>
-    <mergeCell ref="B33:B38"/>
-    <mergeCell ref="C33:C38"/>
-    <mergeCell ref="D9:D11"/>
-    <mergeCell ref="E9:E11"/>
-    <mergeCell ref="D12:D14"/>
-    <mergeCell ref="E12:E14"/>
-    <mergeCell ref="D15:D17"/>
-    <mergeCell ref="E15:E17"/>
-    <mergeCell ref="B9:B14"/>
-    <mergeCell ref="C9:C14"/>
-    <mergeCell ref="B15:B20"/>
-    <mergeCell ref="C15:C20"/>
-    <mergeCell ref="B21:B26"/>
-    <mergeCell ref="C21:C26"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="D3:D5"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="D6:D8"/>
-    <mergeCell ref="E6:E8"/>
-    <mergeCell ref="B3:B8"/>
-    <mergeCell ref="C3:C8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="0" r:id="rId1"/>

</xml_diff>